<commit_message>
Saque la posibilidad de extraer lista de paises para extraer de a un pais.
En el propio df_competencias.xlsx aclaro el nombre del pais y competicion tanto en flashscore como en sofifa (en vez de definirlo dentro de la funcion)
</commit_message>
<xml_diff>
--- a/data_understanding/df_competencias.xlsx
+++ b/data_understanding/df_competencias.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D9BC70-4211-BF4C-B318-171FB205E944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66492BD8-3FAD-EC43-B26F-55DF9DA2C796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="60">
   <si>
     <t>nombre</t>
   </si>
@@ -195,6 +195,27 @@
   </si>
   <si>
     <t>fa community shield</t>
+  </si>
+  <si>
+    <t>espana</t>
+  </si>
+  <si>
+    <t>laliga santander</t>
+  </si>
+  <si>
+    <t>pais_sofifa</t>
+  </si>
+  <si>
+    <t>nombre_sofiifa</t>
+  </si>
+  <si>
+    <t>england</t>
+  </si>
+  <si>
+    <t>spain</t>
+  </si>
+  <si>
+    <t>la liga</t>
   </si>
 </sst>
 </file>
@@ -555,14 +576,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3570E4A9-1B7C-CD4C-90F1-ACEB6414EE21}">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -572,8 +593,14 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -583,8 +610,14 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -594,8 +627,11 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -605,8 +641,11 @@
       <c r="C4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -616,8 +655,11 @@
       <c r="C5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -627,8 +669,11 @@
       <c r="C6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -638,8 +683,11 @@
       <c r="C7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -649,8 +697,11 @@
       <c r="C8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -661,7 +712,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -672,7 +723,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -683,7 +734,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -694,7 +745,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -705,7 +756,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -716,7 +767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -727,7 +778,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -914,7 +965,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -925,7 +976,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -936,7 +987,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -947,7 +998,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -958,7 +1009,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>44</v>
       </c>
@@ -969,7 +1020,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>44</v>
       </c>
@@ -980,7 +1031,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -990,8 +1041,14 @@
       <c r="C39" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D39" t="s">
+        <v>57</v>
+      </c>
+      <c r="E39" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>47</v>
       </c>
@@ -1001,8 +1058,11 @@
       <c r="C40" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D40" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -1012,8 +1072,11 @@
       <c r="C41" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D41" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -1023,8 +1086,11 @@
       <c r="C42" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D42" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -1033,6 +1099,26 @@
       </c>
       <c r="C43" t="s">
         <v>8</v>
+      </c>
+      <c r="D43" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44" t="s">
+        <v>54</v>
+      </c>
+      <c r="C44" t="s">
+        <v>4</v>
+      </c>
+      <c r="D44" t="s">
+        <v>58</v>
+      </c>
+      <c r="E44" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualice el nombre de una columna que estaba mal escrito
</commit_message>
<xml_diff>
--- a/data_understanding/df_competencias.xlsx
+++ b/data_understanding/df_competencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66492BD8-3FAD-EC43-B26F-55DF9DA2C796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE05DD2-AB0F-9248-8D88-FFF6D4A8C4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
@@ -206,9 +206,6 @@
     <t>pais_sofifa</t>
   </si>
   <si>
-    <t>nombre_sofiifa</t>
-  </si>
-  <si>
     <t>england</t>
   </si>
   <si>
@@ -216,6 +213,9 @@
   </si>
   <si>
     <t>la liga</t>
+  </si>
+  <si>
+    <t>nombre_sofifa</t>
   </si>
 </sst>
 </file>
@@ -597,7 +597,7 @@
         <v>55</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -1042,7 +1042,7 @@
         <v>4</v>
       </c>
       <c r="D39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E39" t="s">
         <v>48</v>
@@ -1059,7 +1059,7 @@
         <v>4</v>
       </c>
       <c r="D40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1073,7 +1073,7 @@
         <v>8</v>
       </c>
       <c r="D41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1087,7 +1087,7 @@
         <v>8</v>
       </c>
       <c r="D42" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1101,7 +1101,7 @@
         <v>8</v>
       </c>
       <c r="D43" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1115,13 +1115,14 @@
         <v>4</v>
       </c>
       <c r="D44" t="s">
+        <v>57</v>
+      </c>
+      <c r="E44" t="s">
         <v>58</v>
-      </c>
-      <c r="E44" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>